<commit_message>
minor changes to file and presentation structure
</commit_message>
<xml_diff>
--- a/experiment_stimuli/Block1.xlsx
+++ b/experiment_stimuli/Block1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frances\Desktop\sdt\experiment_stimuli\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EBF13B3-48C7-40BD-A3E2-68FE945599E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94AD32F-252A-4D18-B9D7-D2BDDDE75F58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1800" yWindow="1176" windowWidth="17172" windowHeight="11064" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8034" yWindow="1092" windowWidth="17172" windowHeight="11064" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -70,15 +70,9 @@
     <t>The bird was a large explosion.</t>
   </si>
   <si>
-    <t>The forgotten item was a ketchup.</t>
-  </si>
-  <si>
     <t>The blank paper was a catapult.</t>
   </si>
   <si>
-    <t>The desert storm was a donut.</t>
-  </si>
-  <si>
     <t>Metaphors</t>
   </si>
   <si>
@@ -95,6 +89,12 @@
   </si>
   <si>
     <t>correct_answer</t>
+  </si>
+  <si>
+    <t>The desert storm was a carrot.</t>
+  </si>
+  <si>
+    <t>The forgotten item was purple mustard.</t>
   </si>
 </sst>
 </file>
@@ -380,7 +380,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
@@ -544,7 +544,7 @@
         <v>14</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D11" s="1">
         <v>2</v>
@@ -561,7 +561,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D12" s="1">
         <v>1</v>
@@ -578,7 +578,7 @@
         <v>14</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D13" s="1">
         <v>2</v>
@@ -592,10 +592,10 @@
         <v>1</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>6</v>
@@ -609,10 +609,10 @@
         <v>1</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>6</v>
@@ -626,10 +626,10 @@
         <v>1</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>6</v>
@@ -643,10 +643,10 @@
         <v>1</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>6</v>

</xml_diff>